<commit_message>
feat(F-NAR-019): ATOM-AUT.ROU.001-02 Les miettes de Victorina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.ROU.001-02.xlsx
+++ b/stories/arbres/ATOM-AUT.ROU.001-02.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut dire bonjour à l'oiseau gris. Elle va trop vite, l'oiseau part. Une chose puis la suivante, elle pose des miettes sur la barrière.</t>
+          <t>Victorina veut porter les miettes à l'oiseau de la barrière, maintenant. Un éclat de bec saute sur l'oiseau de bois. Elle prend coupelle et chaussure : les miettes tombent, l'oiseau part. Elle refuse de foncer, pull puis pain, puis le jardin. Le vent emporte le tas ; elle pose une à une, suit l'éclat. L'éclat de bec tient le soleil.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau gris tape la vitre. Toc. Toc. Il a un ventre tout rond. Il penche la tête. Dehors, l'herbe est mouillée. Une goutte brille sur une feuille. Le ciel est rose, tout pâle. Une branche frotte le mur, tout bas. Le jardin sent la rosée. Victorina, tu entends l'oiseau ? Oui, maman. Il chante. Il dit bonjour. En ce moment, Victorina ouvre les yeux. Le drap jaune est chaud. Ça sent le linge propre. Je veux le voir. Victorina va vers la fenêtre. Elle est encore en chemise de nuit. L'oiseau s'envole vers la barrière. Il part. Il va au jardin. Nous aussi, tout à l'heure. D'abord le matin. Une chose, puis la suivante. Victorina pose la main sur la vitre. La vitre est un peu froide. Le rideau blanc bouge très peu. On se lève ? Oui. Victorina quitte le drap. Ses pieds touchent le tapis. Le tapis est doux. Le pull, maintenant.</t>
+          <t>La coupelle jaune a passé la nuit. Des miettes sèches y tiennent. À côté, un oiseau de bois. Son bec capte un bout de soleil. Un éclat de bec saute sur le bois. Le rideau jaune bouge un peu. Une chaise attend le pull vert. Victorina ouvre un œil. Le drap jaune est chaud. Ça sent le linge propre. Dehors, l'herbe brille, un peu froide. La barrière ronde attend au fond. Victorina, tu vois l'oiseau dehors ? Oui, papa. Il est sur la barrière ! Il a faim, je crois. Je lui porte les miettes maintenant ! Le pain est à la cuisine. En ce moment, Victorina saute du lit. Elle est en chemise de nuit. Ses pieds touchent le tapis. Le tapis est chaud, un peu rêche. C'est pour lui ! Victorina saisit la coupelle d'une main. De l'autre, elle attrape une chaussure. Le pull, aussi. Elle penche vers le pull vert. La coupelle bascule. Les miettes tombent sur le tapis. Oh non ! Dehors, l'oiseau s'envole. Il part ! Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Papa s'accroupit à la même hauteur. Tu veux courir, ou regarder ? Je veux l'oiseau. Victorina baisse les épaules. Les miettes sont là, au sol.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau gris tape la vitre. Toc. Toc. Il a un ventre tout rond. Il penche la tête. Dehors, l'herbe est mouillée. Une goutte brille sur une feuille. Le ciel est rose, tout pâle. Une branche frotte le mur, tout bas. Le jardin sent la rosée. Victorina, tu entends l'oiseau ? Oui, maman. Il chante. Il dit bonjour. En ce moment, Victorina ouvre les yeux. Le drap jaune est chaud. Ça sent le linge propre. Je veux le voir. Victorina va vers la fenêtre. Elle est encore en chemise de nuit. L'oiseau s'envole vers la barrière. Il part. Il va au jardin. Nous aussi, tout à l'heure. D'abord le matin. Une chose, puis la suivante. Victorina pose la main sur la vitre. La vitre est un peu froide. Le rideau blanc bouge très peu. On se lève ? Oui. Victorina quitte le drap. Ses pieds touchent le tapis. Le tapis est doux. Le pull, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La coupelle jaune a passé la nuit. Des miettes sèches y tiennent. À côté, un oiseau de bois. Son bec capte un bout de soleil. Un &lt;emphasis level="moderate"&gt;éclat de bec&lt;/emphasis&gt; saute sur le bois. Le rideau jaune bouge un peu. Une chaise attend le pull vert. Victorina ouvre un œil. Le drap jaune est chaud. Ça sent le linge propre. Dehors, l'herbe brille, un peu froide. La barrière ronde attend au fond. Victorina, tu vois l'oiseau dehors ? Oui, papa. Il est sur la barrière ! Il a faim, je crois. Je lui porte les miettes maintenant ! Le pain est à la cuisine. En ce moment, Victorina saute du lit. Elle est en chemise de nuit. Ses pieds touchent le tapis. Le tapis est chaud, un peu rêche. C'est pour lui ! Victorina saisit la coupelle d'une main. De l'autre, elle attrape une chaussure. Le pull, aussi. Elle penche vers le pull vert. La coupelle bascule. Les miettes tombent sur le tapis. Oh non ! Dehors, l'oiseau s'envole. Il part ! Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Papa s'accroupit à la même hauteur. Tu veux courir, ou regarder ? Je veux l'oiseau. Victorina baisse les épaules. Les miettes sont là, au sol.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le soleil entre. Lila ouvre les yeux. Maman dit : c'est le matin. &lt;emphasis&gt;une&lt;/emphasis&gt; étape après l'autre. D'abord, Lila se lève. Ses pieds touchent le tapis. Ensuite, Lila s'habille. Elle met le pull. Elle met le pantalon. Papa dit : maintenant, le déjeuner. Lila s'assoit. Elle mange du pain. Elle boit du lait. Maman dit : ensuite, le sac. Lila met la gourde. Lila met le doudou. Une étape après l'autre. Lila est prête.&lt;/slow&gt; [pause]</t>
+          <t>La coupelle jaune a passé la nuit. Des miettes sèches y tiennent. À côté, un oiseau de bois. Son bec capte un bout de soleil. Un &lt;emphasis&gt;éclat de bec&lt;/emphasis&gt; saute sur le bois. Le rideau jaune bouge un peu. Une chaise attend le pull vert. Victorina ouvre un œil. Le drap jaune est chaud. Ça sent le linge propre. Dehors, l'herbe brille, un peu froide. La barrière ronde attend au fond. Victorina, tu vois l'oiseau dehors ? Oui, papa. Il est sur la barrière ! Il a faim, je crois. Je lui porte les miettes maintenant ! Le pain est à la cuisine. En ce moment, Victorina saute du lit. Elle est en chemise de nuit. Ses pieds touchent le tapis. Le tapis est chaud, un peu rêche. C'est pour lui ! Victorina saisit la coupelle d'une main. De l'autre, elle attrape une chaussure. Le pull, aussi. Elle penche vers le pull vert. La coupelle bascule. Les miettes tombent sur le tapis. Oh non ! Dehors, l'oiseau s'envole. Il part ! Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Papa s'accroupit à la même hauteur. Tu veux courir, ou regarder ? Je veux l'oiseau. Victorina baisse les épaules. Les miettes sont là, au sol. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de bec</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,46 +1319,55 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=l_eclat_de_bec_sur_l_oiseau_de_bois; tempo=naturel; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un oiseau gris tape la vitre.
-narrateur|Toc.
-narrateur|Toc.
-narrateur|Il a un ventre tout rond.
-narrateur|Il penche la tête.
-narrateur|Dehors, l'herbe est mouillée.
-narrateur|Une goutte brille sur une feuille.
-narrateur|Le ciel est rose, tout pâle.
-narrateur|Une branche frotte le mur, tout bas.
-narrateur|Le jardin sent la rosée.
-maman|Victorina, tu entends l'oiseau ?
-enfant-f|Oui, maman.
-enfant-f|Il chante.
-papa|Il dit bonjour.
-narrateur|En ce moment, Victorina ouvre les yeux.
+          <t>narrateur|La coupelle jaune a passé la nuit.
+narrateur|Des miettes sèches y tiennent.
+narrateur|À côté, un oiseau de bois.
+narrateur|Son bec capte un bout de soleil.
+narrateur|Un éclat de bec saute sur le bois.
+narrateur|Le rideau jaune bouge un peu.
+narrateur|Une chaise attend le pull vert.
+narrateur|Victorina ouvre un œil.
 narrateur|Le drap jaune est chaud.
 narrateur|Ça sent le linge propre.
-enfant-f|Je veux le voir.
-narrateur|Victorina va vers la fenêtre.
-narrateur|Elle est encore en chemise de nuit.
-narrateur|L'oiseau s'envole vers la barrière.
-enfant-f|Il part.
-maman|Il va au jardin.
-papa|Nous aussi, tout à l'heure.
-maman|D'abord le matin.
-maman|Une chose, puis la suivante.
-narrateur|Victorina pose la main sur la vitre.
-narrateur|La vitre est un peu froide.
-narrateur|Le rideau blanc bouge très peu.
-papa|On se lève ?
-enfant-f|Oui.
-narrateur|Victorina quitte le drap.
+narrateur|Dehors, l'herbe brille, un peu froide.
+narrateur|La barrière ronde attend au fond.
+papa|Victorina, tu vois l'oiseau dehors ?
+enfant-f|Oui, papa.
+enfant-f|Il est sur la barrière !
+maman|Il a faim, je crois.
+enfant-f|Je lui porte les miettes maintenant !
+papa|Le pain est à la cuisine.
+narrateur|En ce moment, Victorina saute du lit.
+narrateur|Elle est en chemise de nuit.
 narrateur|Ses pieds touchent le tapis.
-narrateur|Le tapis est doux.
-papa|Le pull, maintenant.</t>
+narrateur|Le tapis est chaud, un peu rêche.
+enfant-f|C'est pour lui !
+narrateur|Victorina saisit la coupelle d'une main.
+narrateur|De l'autre, elle attrape une chaussure.
+maman|Le pull, aussi.
+narrateur|Elle penche vers le pull vert.
+narrateur|La coupelle bascule.
+narrateur|Les miettes tombent sur le tapis.
+enfant-f|Oh non !
+narrateur|Dehors, l'oiseau s'envole.
+enfant-f|Il part !
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux courir, ou regarder ?
+enfant-f|Je veux l'oiseau.
+narrateur|Victorina baisse les épaules.
+maman|Les miettes sont là, au sol.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1390,27 +1399,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorina veut l'oiseau. Comment se prépare-t-elle ?</t>
+          <t>Victorina veut porter les miettes. Où sont-elles tombées ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina veut l'oiseau. Comment se prépare-t-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina veut porter les &lt;emphasis level="moderate"&gt;miettes&lt;/emphasis&gt;. Où sont-elles tombées ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lila se prépare. Comment avance-t-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina veut porter les &lt;emphasis&gt;miettes&lt;/emphasis&gt;. Où sont-elles tombées ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>une chose</t>
+          <t>le tapis</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>une chose | puis l'autre | d'abord | doucement | une chose puis l'autre | puis la suivante</t>
+          <t>le tapis | tapis | par terre | au sol | sur le tapis | tombées</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1425,7 +1434,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle fait une chose, puis la suivante. Comment se prépare Victorina ?</t>
+          <t>La coupelle a basculé. Où sont les miettes ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1463,7 +1472,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1471,10 +1480,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1489,34 +1498,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>miettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1525,13 +1538,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1541,13 +1554,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les_miettes_sont_sur_le_tapis; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorina veut l'oiseau.
-narrateur|Comment se prépare-t-elle ?</t>
+          <t>narrateur|Victorina veut porter les miettes.
+maman|Où sont-elles tombées ?</t>
         </is>
       </c>
     </row>
@@ -1574,17 +1587,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le pull vert, sur la chaise. Victorina enfile le pull. Le pull sent le jardin, un peu. C'est vert, comme l'herbe. Oui. Ensuite, le pain. Victorina va à la cuisine. Le carrelage est froid. La table est déjà mise. Tu veux le pain d'abord ? Le pain. Elle s'assoit. Elle croque un bout de pain. Le pain est un peu dur. On garde une miette ? Pour l'oiseau. Oui. Dans ta main, tout doux. Merci, Victorina.</t>
+          <t>J'arrête de tout prendre. Elle pose la chaussure près du lit. Elle ramasse trois miettes, sans se presser. Vous attendez. Le pull vert est sur la chaise. Tu le mets ? Oui, papa. Victorina enfile le pull. Le pull sent un peu le jardin. C'est vert, comme l'herbe. Le pain t'attend, à table. Victorina va vers la cuisine. Le carrelage est froid sous ses pieds. La table sent le pain chaud. Un bol bleu attend près du pain. Tu manges un bout, d'abord ? Le pain. Elle s'assoit. Elle croque un coin de pain. Le pain est un peu dur. Une miette reste au bord. On garde des miettes ? Pour l'oiseau. Dans la coupelle jaune. Victorina glisse les miettes dedans. Sur la commode, l'éclat de bec brille. Il me montre le jardin. Elle respire, un peu. Les chaussures, après. Oui.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le pull vert, sur la chaise. Victorina enfile le pull. Le pull sent le jardin, un peu. C'est vert, comme l'herbe. Oui. Ensuite, le pain. Victorina va à la cuisine. Le carrelage est froid. La table est déjà mise. Tu veux le pain d'abord ? Le pain. Elle s'assoit. Elle croque un bout de pain. Le pain est un peu dur. On garde une miette ? Pour l'oiseau. Oui. Dans ta main, tout doux. Merci, Victorina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'arrête de tout prendre. Elle pose la chaussure près du lit. Elle ramasse trois miettes, sans se presser. Vous attendez. Le pull vert est sur la chaise. Tu le mets ? Oui, papa. Victorina enfile le pull. Le pull sent un peu le jardin. C'est vert, comme l'herbe. Le pain t'attend, à table. Victorina va vers la cuisine. Le carrelage est froid sous ses pieds. La table sent le pain chaud. Un bol bleu attend près du pain. Tu manges un bout, d'abord ? Le pain. Elle s'assoit. Elle croque un coin de pain. Le pain est un peu dur. Une miette reste au bord. On garde des miettes ? Pour l'oiseau. Dans la coupelle jaune. Victorina glisse les miettes dedans. Sur la commode, l'&lt;emphasis level="moderate"&gt;éclat de bec&lt;/emphasis&gt; brille. Il me montre le jardin. Elle respire, un peu. Les chaussures, après. Oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lila a fait l'étape dite. Se lever. S'habiller. Déje&lt;emphasis&gt;une&lt;/emphasis&gt;r. Le sac. Une étape après l'autre.&lt;/slow&gt; [pause]</t>
+          <t>J'arrête de tout prendre. Elle pose la chaussure près du lit. Elle ramasse trois miettes, sans se presser. Vous attendez. Le pull vert est sur la chaise. Tu le mets ? Oui, papa. Victorina enfile le pull. Le pull sent un peu le jardin. C'est vert, comme l'herbe. Le pain t'attend, à table. Victorina va vers la cuisine. Le carrelage est froid sous ses pieds. La table sent le pain chaud. Un bol bleu attend près du pain. Tu manges un bout, d'abord ? Le pain. Elle s'assoit. Elle croque un coin de pain. Le pain est un peu dur. Une miette reste au bord. On garde des miettes ? Pour l'oiseau. Dans la coupelle jaune. Victorina glisse les miettes dedans. Sur la commode, l'&lt;emphasis&gt;éclat de bec&lt;/emphasis&gt; brille. Il me montre le jardin. Elle respire, un peu. Les chaussures, après. Oui. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1631,7 +1644,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1639,10 +1652,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1665,30 +1678,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de bec</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1697,10 +1710,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1709,34 +1722,50 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=pull_puis_pain_puis_miettes; tempo=naturel; sourire=franc; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>papa|Le pull vert, sur la chaise.
+          <t>enfant-f|J'arrête de tout prendre.
+narrateur|Elle pose la chaussure près du lit.
+narrateur|Elle ramasse trois miettes, sans se presser.
+enfant-f|Vous attendez.
+narrateur|Le pull vert est sur la chaise.
+papa|Tu le mets ?
+enfant-f|Oui, papa.
 narrateur|Victorina enfile le pull.
-narrateur|Le pull sent le jardin, un peu.
+narrateur|Le pull sent un peu le jardin.
 enfant-f|C'est vert, comme l'herbe.
-maman|Oui.
-maman|Ensuite, le pain.
-narrateur|Victorina va à la cuisine.
-narrateur|Le carrelage est froid.
-narrateur|La table est déjà mise.
-maman|Tu veux le pain d'abord ?
+maman|Le pain t'attend, à table.
+narrateur|Victorina va vers la cuisine.
+narrateur|Le carrelage est froid sous ses pieds.
+narrateur|La table sent le pain chaud.
+narrateur|Un bol bleu attend près du pain.
+maman|Tu manges un bout, d'abord ?
 enfant-f|Le pain.
 narrateur|Elle s'assoit.
-narrateur|Elle croque un bout de pain.
+narrateur|Elle croque un coin de pain.
 narrateur|Le pain est un peu dur.
-maman|On garde une miette ?
+narrateur|Une miette reste au bord.
+maman|On garde des miettes ?
 enfant-f|Pour l'oiseau.
-papa|Oui.
-papa|Dans ta main, tout doux.
-maman|Merci, Victorina.</t>
+papa|Dans la coupelle jaune.
+narrateur|Victorina glisse les miettes dedans.
+narrateur|Sur la commode, l'éclat de bec brille.
+enfant-f|Il me montre le jardin.
+narrateur|Elle respire, un peu.
+papa|Les chaussures, après.
+enfant-f|Oui.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pain</t>
         </is>
       </c>
     </row>
@@ -1763,17 +1792,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ensuite, le sac. Le sac rouge attend près du banc. Victorina met la gourde. Elle met le doudou. Les miettes, avec nous. Dans ma main. Victorina met ses chaussures. Les chaussures sont un peu serrées. On les ajuste ? Oui. Papa ouvre la porte. L'air sent le jardin. L'herbe brille encore. L'oiseau est sur la barrière. Il est là ! Pose les miettes. Victorina pose les miettes. L'oiseau penche la tête. Il picore une miette. Puis une autre. Il dit merci. On reste un peu, tout calmes. Il a le ventre rond. Une goutte brille encore sur la feuille. L'herbe est froide sous les chaussures. Tu lui as dit bonjour ? Oui, tout doux.</t>
+          <t>Victorina enfile les deux chaussures. Elles serrent un peu. On les ajuste ? Oui. Papa ouvre la porte. L'air sent l'herbe mouillée. La barrière ronde est vide. Il n'est plus là ! Victorina court vers le banc. Elle verse les miettes d'un coup. Le vent les emporte dans l'herbe. Elles partent ! La coupelle est vide. Le sourire ne revient pas. Pas comme ça. Elle refuse de foncer. Elle reste près du banc. Personne ne parle. Un petit oiseau gris revient. Il se pose sur la barrière. Sur son bec, un éclat de bec. Comme sur le bois ! Tu le vois, toi ? Victorina pose trois miettes, une à une. L'oiseau penche la tête. Il picore une miette. Il dit merci. Merci d'avoir posé, Victorina. La coupelle reste sur le banc.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ensuite, le sac. Le sac rouge attend près du banc. Victorina met la gourde. Elle met le doudou. Les miettes, avec nous. Dans ma main. Victorina met ses chaussures. Les chaussures sont un peu serrées. On les ajuste ? Oui. Papa ouvre la porte. L'air sent le jardin. L'herbe brille encore. L'oiseau est sur la barrière. Il est là ! Pose les miettes. Victorina pose les miettes. L'oiseau penche la tête. Il picore une miette. Puis une autre. Il dit merci. On reste un peu, tout calmes. Il a le ventre rond. Une goutte brille encore sur la feuille. L'herbe est froide sous les chaussures. Tu lui as dit bonjour ? Oui, tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorina enfile les deux chaussures. Elles serrent un peu. On les ajuste ? Oui. Papa ouvre la porte. L'air sent l'herbe mouillée. La barrière ronde est vide. Il n'est plus là ! Victorina court vers le banc. Elle verse les miettes d'un coup. Le vent les emporte dans l'herbe. Elles partent ! La coupelle est vide. Le sourire ne revient pas. Pas comme ça. Elle refuse de foncer. Elle reste près du banc. Personne ne parle. Un petit oiseau gris revient. Il se pose sur la barrière. Sur son bec, un &lt;emphasis level="moderate"&gt;éclat de bec&lt;/emphasis&gt;. Comme sur le bois ! Tu le vois, toi ? Victorina pose trois miettes, une à une. L'oiseau penche la tête. Il picore une miette. Il dit merci. Merci d'avoir posé, Victorina. La coupelle reste sur le banc.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lila met les chaussures. Papa ouvre la porte.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Victorina enfile les deux chaussures. Elles serrent un peu. On les ajuste ? Oui. Papa ouvre la porte. L'air sent l'herbe mouillée. La barrière ronde est vide. Il n'est plus là ! Victorina court vers le banc. Elle verse les miettes d'un coup. Le vent les emporte dans l'herbe. Elles partent ! La coupelle est vide. Le sourire ne revient pas. Pas comme ça. Elle refuse de foncer. Elle reste près du banc. Personne ne parle. Un petit oiseau gris revient. Il se pose sur la barrière. Sur son bec, un &lt;emphasis&gt;éclat de bec&lt;/emphasis&gt;. Comme sur le bois ! Tu le vois, toi ? Victorina pose trois miettes, une à une. L'oiseau penche la tête. Il picore une miette. Il dit merci. Merci d'avoir posé, Victorina. La coupelle reste sur le banc.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1820,7 +1849,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1828,22 +1857,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1852,28 +1885,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de bec</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1882,55 +1919,61 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=deux_envies_qui_se_heurtent; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_bec; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|Ensuite, le sac.
-narrateur|Le sac rouge attend près du banc.
-narrateur|Victorina met la gourde.
-narrateur|Elle met le doudou.
-papa|Les miettes, avec nous.
-enfant-f|Dans ma main.
-narrateur|Victorina met ses chaussures.
-narrateur|Les chaussures sont un peu serrées.
+          <t>narrateur|Victorina enfile les deux chaussures.
+narrateur|Elles serrent un peu.
 papa|On les ajuste ?
 enfant-f|Oui.
 narrateur|Papa ouvre la porte.
-narrateur|L'air sent le jardin.
-narrateur|L'herbe brille encore.
-narrateur|L'oiseau est sur la barrière.
-enfant-f|Il est là !
-maman|Pose les miettes.
-narrateur|Victorina pose les miettes.
+narrateur|L'air sent l'herbe mouillée.
+narrateur|La barrière ronde est vide.
+enfant-f|Il n'est plus là !
+narrateur|Victorina court vers le banc.
+narrateur|Elle verse les miettes d'un coup.
+narrateur|Le vent les emporte dans l'herbe.
+enfant-f|Elles partent !
+narrateur|La coupelle est vide.
+narrateur|Le sourire ne revient pas.
+enfant-f|Pas comme ça.
+narrateur|Elle refuse de foncer.
+narrateur|Elle reste près du banc.
+narrateur|Personne ne parle.
+narrateur|Un petit oiseau gris revient.
+narrateur|Il se pose sur la barrière.
+narrateur|Sur son bec, un éclat de bec.
+enfant-f|Comme sur le bois !
+papa|Tu le vois, toi ?
+narrateur|Victorina pose trois miettes, une à une.
 narrateur|L'oiseau penche la tête.
 narrateur|Il picore une miette.
-narrateur|Puis une autre.
-papa|Il dit merci.
-maman|On reste un peu, tout calmes.
-enfant-f|Il a le ventre rond.
-narrateur|Une goutte brille encore sur la feuille.
-narrateur|L'herbe est froide sous les chaussures.
-maman|Tu lui as dit bonjour ?
-enfant-f|Oui, tout doux.</t>
+enfant-f|Il dit merci.
+papa|Merci d'avoir posé, Victorina.
+narrateur|La coupelle reste sur le banc.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte</t>
+          <t>porte,oiseau</t>
         </is>
       </c>
     </row>
@@ -1957,17 +2000,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Bonjour, oiseau. Tu as avancé tout doucement. Une chose, puis la suivante. L'oiseau picore encore. Bravo, Victorina. Le ventre rond brille au soleil.</t>
+          <t>L'oiseau picore près du banc. Bonjour, oiseau. Tu lui as porté les miettes ? Oui, maman. La coupelle jaune reste sur le bois. Une miette colle au banc. L'éclat de bec reste sur le bec. Il brille. Victorina serre le pull contre elle. Le jardin sent l'herbe froide. On reste un peu ? Oui, papa. L'éclat de bec tient le soleil.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Bonjour, oiseau. Tu as avancé tout doucement. Une chose, puis la suivante. L'oiseau picore encore. Bravo, Victorina. Le ventre rond brille au soleil.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oiseau picore près du banc. Bonjour, oiseau. Tu lui as porté les miettes ? Oui, maman. La coupelle jaune reste sur le bois. Une miette colle au banc. L'&lt;emphasis level="moderate"&gt;éclat de bec&lt;/emphasis&gt; reste sur le bec. Il brille. Victorina serre le pull contre elle. Le jardin sent l'herbe froide. On reste un peu ? Oui, papa. L'éclat de bec tient le soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oiseau picore près du banc. Bonjour, oiseau. Tu lui as porté les miettes ? Oui, maman. La coupelle jaune reste sur le bois. Une miette colle au banc. L'&lt;emphasis&gt;éclat de bec&lt;/emphasis&gt; reste sur le bec. Il brille. Victorina serre le pull contre elle. Le jardin sent l'herbe froide. On reste un peu ? Oui, papa. L'éclat de bec tient le soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2014,18 +2057,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2034,12 +2077,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2048,17 +2091,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de bec</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2067,11 +2114,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2080,29 +2127,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_bec_tient_le_soleil; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Bonjour, oiseau.
-maman|Tu as avancé tout doucement.
-papa|Une chose, puis la suivante.
-narrateur|L'oiseau picore encore.
-papa|Bravo, Victorina.
-narrateur|Le ventre rond brille au soleil.</t>
+          <t>narrateur|L'oiseau picore près du banc.
+enfant-f|Bonjour, oiseau.
+maman|Tu lui as porté les miettes ?
+enfant-f|Oui, maman.
+narrateur|La coupelle jaune reste sur le bois.
+narrateur|Une miette colle au banc.
+narrateur|L'éclat de bec reste sur le bec.
+enfant-f|Il brille.
+narrateur|Victorina serre le pull contre elle.
+narrateur|Le jardin sent l'herbe froide.
+papa|On reste un peu ?
+enfant-f|Oui, papa.
+narrateur|L'éclat de bec tient le soleil.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>oiseau</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2215,6 +2278,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>